<commit_message>
Rebased epochs to 2
</commit_message>
<xml_diff>
--- a/hyperparam_base_2.xlsx
+++ b/hyperparam_base_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\AMLS2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E74E00-D710-49AA-B961-5194B27DC14E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AC173E5-689D-43A1-A877-348FAB4A4A8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2985" yWindow="4350" windowWidth="38700" windowHeight="15075" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -505,7 +505,7 @@
         <v>2</v>
       </c>
       <c r="C2">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s">
         <v>10</v>

</xml_diff>